<commit_message>
new pages and test cases added
</commit_message>
<xml_diff>
--- a/src/test/resources/automationpracticeproject.xlsx
+++ b/src/test/resources/automationpracticeproject.xlsx
@@ -9,11 +9,14 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="signup" sheetId="1" r:id="rId1"/>
     <sheet name="accountInformation" sheetId="2" r:id="rId2"/>
+    <sheet name="logoutuser" sheetId="3" r:id="rId3"/>
+    <sheet name="loginuser" sheetId="4" r:id="rId4"/>
+    <sheet name="contactUsForm" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="29">
   <si>
     <t>Name</t>
   </si>
@@ -94,6 +97,24 @@
   </si>
   <si>
     <t>sannn@med.com</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>textarea</t>
+  </si>
+  <si>
+    <t>subject</t>
+  </si>
+  <si>
+    <t xml:space="preserve">learning java and selenium for automation testing </t>
+  </si>
+  <si>
+    <t>contact us form</t>
   </si>
 </sst>
 </file>
@@ -552,4 +573,173 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="3">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1992</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K2" s="3">
+        <v>635852</v>
+      </c>
+      <c r="L2" s="3">
+        <v>8456978945</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.140625" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" customWidth="1"/>
+    <col min="3" max="3" width="48.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>